<commit_message>
uploaded updated database and publisher with cache busting
</commit_message>
<xml_diff>
--- a/tools/resource-publisher/GenAI-Hub-Resource-Database.xlsx
+++ b/tools/resource-publisher/GenAI-Hub-Resource-Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/willcrook/Documents/Code Projects/GenAI-Hub/tools/resource-publisher/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B750E09-A690-2344-A758-B55054B03CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F11C2CE-9E29-924F-B37E-6319C86D4D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Showcases" sheetId="10" r:id="rId1"/>
@@ -1378,7 +1378,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="235">
   <si>
     <t>id</t>
   </si>
@@ -2084,6 +2084,9 @@
   <si>
     <t>University Provided|Web search grounding | Integration with Office Tools</t>
   </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;url=https%3A%2F%2Fen.wikiversity.org%2Fwiki%2FArtificial_intelligence&amp;ved=0CBYQjRxqFwoTCOCfvaa35pUDFQAAAAAdAAAAABBS&amp;opi=89978449</t>
+  </si>
 </sst>
 </file>
 
@@ -2093,7 +2096,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2107,6 +2110,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2149,10 +2160,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2176,8 +2188,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
@@ -2574,9 +2590,9 @@
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0700-00000D000000}" name="featured"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="published"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0700-00000F000000}" name="estimated_minutes"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="thumbnail_src"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="thumbnail_src" dataCellStyle="Hyperlink"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="thumbnail_alt"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="file_url"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0700-000012000000}" name="file_url" dataCellStyle="Hyperlink"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="file_name"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="file_format"/>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0700-000015000000}" name="file_size_bytes"/>
@@ -30970,16 +30986,18 @@
       <c r="L2" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="M2" s="2" t="b">
-        <v>0</v>
+      <c r="M2" s="2" t="s">
+        <v>209</v>
       </c>
       <c r="N2" s="2" t="b">
         <v>1</v>
       </c>
       <c r="O2" s="6"/>
-      <c r="P2" s="2"/>
+      <c r="P2" s="11" t="s">
+        <v>234</v>
+      </c>
       <c r="Q2" s="2"/>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="11" t="s">
         <v>135</v>
       </c>
       <c r="S2" s="2" t="s">
@@ -34025,10 +34043,14 @@
       <formula1>OR(U2="",AND(ISNUMBER(U2),U2&gt;=0,U2=INT(U2)))</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="R2" r:id="rId1" xr:uid="{4FFCA5BC-F05A-6643-85FC-1E468C31C6D6}"/>
+    <hyperlink ref="P2" r:id="rId2" xr:uid="{3003D97D-698A-284C-98F6-3924E60E61B9}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>